<commit_message>
mark2publish covered with test
</commit_message>
<xml_diff>
--- a/htdocs/tests/Cases/Integration/files/cetaf_sid.xlsx
+++ b/htdocs/tests/Cases/Integration/files/cetaf_sid.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="33">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -116,6 +116,9 @@
   </si>
   <si>
     <t xml:space="preserve">Černošice - Praha-Západ: Na okraji pole u obce Černošice - Nová Vráž. 15 km JZ Prahy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEST_5</t>
   </si>
 </sst>
 </file>
@@ -322,7 +325,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr defaultColWidth="19.61328125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="14" min="1" style="1" width="19.61"/>
@@ -483,6 +486,41 @@
         <v>2017</v>
       </c>
       <c r="N4" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="M5" s="1" t="n">
+        <v>2017</v>
+      </c>
+      <c r="N5" s="1" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>